<commit_message>
Table and chain: single round-UP (ceiling) at the final integer mA so a reading is never below the true current; spec and tests updated; Program Map regenerated
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Documentation/Program_Map.xlsx
+++ b/Documentation/Program_Map.xlsx
@@ -1220,7 +1220,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>735</t>
+          <t>734</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -4445,7 +4445,7 @@
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>508</t>
+          <t>507</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -4472,12 +4472,12 @@
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>444</t>
+          <t>442</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>قالب فرمول مشترک هر دو کانال، یک مرحله برای هر المان شماتیک: شمارش -&gt; mV پایه ADC -&gt; خنثی‌کردن تقسیم ‎R41/R42 -&gt;‎ خنثی‌کردن گین LM358 -&gt; خنثی‌کردن mΩ شانت -&gt; mA، سپس آفست صفر پر-کانال و گین پرمیل بنچ. هر ضرب مرحلهٔ صورت/مخرج خودش را جابه‌جا می‌کند و فقط یک تقسیم در انتها اجرا می‌شود. رژیم فلش: پنج مرحله در یک ضرب+تقسیم 32بیتی با نتیجهٔ بیت‌به‌بیت یکسان جمع شد (اثبات برای هر 4096 شمارش؛ تقسیم 64بیتی ~1KB می‌خواست). اگر مقاومتی عوض شد دوباره اشتقاق بگیر (تست هاست از همین دیفاین‌ها بازمحاسبه می‌کند). رُند: تقسیم جمع‌شده همان قاعدهٔ رُند به نزدیکِ پنل و لنگرهای جدول بنچ را دارد (نصف مقسوم‌علیه پیش از تقسیم)، چون زنجیرهٔ برشی، کم‌خوانی یک‌طرفهٔ جریان اندازه‌گیری‌شده است.</t>
+          <t>قالب فرمول مشترک هر دو کانال، یک مرحله برای هر المان شماتیک: شمارش -&gt; mV پایه ADC -&gt; خنثی‌کردن تقسیم ‎R41/R42 -&gt;‎ خنثی‌کردن گین LM358 -&gt; خنثی‌کردن mΩ شانت -&gt; mA، سپس آفست صفر پر-کانال و گین پرمیل بنچ. هر ضرب مرحلهٔ صورت/مخرج خودش را جابه‌جا می‌کند و فقط یک تقسیم در انتها اجرا می‌شود. رژیم فلش: پنج مرحله در یک ضرب+تقسیم 32بیتی با نتیجهٔ بیت‌به‌بیت یکسان جمع شد (اثبات برای هر 4096 شمارش؛ تقسیم 64بیتی ~1KB می‌خواست). اگر مقاومتی عوض شد دوباره اشتقاق بگیر (تست هاست از همین دیفاین‌ها بازمحاسبه می‌کند). رُند: تقسیم جمع‌شده رو به بالا (سقف) گرد می‌شود، همان قاعدهٔ درون‌یابی جدول؛ هیچ گرد یا برشی‌ای نباید از جریان واقعی پایین‌تر بخواند.</t>
         </is>
       </c>
     </row>
@@ -4499,7 +4499,7 @@
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>529</t>
+          <t>528</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -4553,7 +4553,7 @@
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>574</t>
+          <t>573</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -4580,7 +4580,7 @@
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>545</t>
+          <t>544</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -4607,7 +4607,7 @@
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>591</t>
+          <t>590</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -4634,7 +4634,7 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>554</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -4661,7 +4661,7 @@
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>731</t>
+          <t>730</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>694</t>
+          <t>693</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -4715,7 +4715,7 @@
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>678</t>
+          <t>677</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>485</t>
+          <t>483</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -4769,7 +4769,7 @@
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>644</t>
+          <t>643</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -4796,7 +4796,7 @@
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>613</t>
+          <t>612</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">

</xml_diff>